<commit_message>
Switch import image references from UUID to title-based matching
Admin now writes the image title (e.g. 'Beach Shot 1') in the Mapping
sheet instead of a 36-char UUID. The import API resolves titles to IDs
case-insensitively before inserting; UUIDs still accepted as fallback.

Updated template, API template route, and imports page instructions.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/imports/whitedoor-import-template.xlsx
+++ b/imports/whitedoor-import-template.xlsx
@@ -484,9 +484,9 @@
   <dimension ref="A1:D4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="40.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,10 +508,10 @@
         <v>R1</v>
       </c>
       <c r="B2" t="str">
-        <v>PASTE-IMAGE-UUID-1</v>
+        <v>Beach Shot 1</v>
       </c>
       <c r="C2" t="str">
-        <v>PASTE-IMAGE-UUID-2</v>
+        <v>Group Photo</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -522,7 +522,7 @@
         <v>R2</v>
       </c>
       <c r="B3" t="str">
-        <v>PASTE-IMAGE-UUID-3</v>
+        <v>Event Highlight</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -536,13 +536,13 @@
         <v>R3</v>
       </c>
       <c r="B4" t="str">
-        <v>PASTE-IMAGE-UUID-4</v>
+        <v>Venue Entrance</v>
       </c>
       <c r="C4" t="str">
-        <v>PASTE-IMAGE-UUID-5</v>
+        <v>Stage Moment</v>
       </c>
       <c r="D4" t="str">
-        <v>PASTE-IMAGE-UUID-6</v>
+        <v>Closing Shot</v>
       </c>
     </row>
   </sheetData>
@@ -554,12 +554,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <cols>
     <col min="1" max="1" width="55.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="70.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -574,280 +574,285 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>HOW TO USE THIS FILE</v>
+        <v>STEP-BY-STEP</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>1. Fill in the Reviews sheet — one row per review.</v>
+        <v>1. Upload your photos first in Admin → Images. Give each one a clear title (e.g. 'Beach Shot 1').</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2. Fill in the Mapping sheet — only for reviews that should include photos.</v>
+        <v>2. Fill in the Reviews sheet — one row per review.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3. Upload this file in Admin → Imports.</v>
+        <v>3. Fill in the Mapping sheet — only for reviews that should include photos.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v xml:space="preserve">   In image_1 / image_2 / image_3, write the TITLE of the photo (not a UUID).</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>── SHEET: Reviews (required) ──────────────────────────────────────────</v>
+        <v>4. Upload this file in Admin → Imports.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Column</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Required?</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Description</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Example</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>local_id</v>
-      </c>
-      <c r="B10" t="str">
-        <v>YES</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Your own reference key. Used to link rows in the Mapping sheet. Any text works.</v>
-      </c>
-      <c r="D10" t="str">
-        <v>R1</v>
+        <v>── SHEET: Reviews (required) ──────────────────────────────────────────</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>event_id</v>
+        <v>Column</v>
       </c>
       <c r="B11" t="str">
-        <v>YES</v>
+        <v>Required?</v>
       </c>
       <c r="C11" t="str">
-        <v>UUID of an event from your Supabase events table. Use the word 'general' (lowercase) for homepage general reviews.</v>
+        <v>Description</v>
       </c>
       <c r="D11" t="str">
-        <v>3f2a1b4c-… OR general</v>
+        <v>Example</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>review_text</v>
+        <v>local_id</v>
       </c>
       <c r="B12" t="str">
         <v>YES</v>
       </c>
       <c r="C12" t="str">
-        <v>The full review text. Keep it genuine and specific.</v>
+        <v>Your own reference key. Used to link rows in the Mapping sheet.</v>
       </c>
       <c r="D12" t="str">
-        <v>Amazing experience…</v>
+        <v>R1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v/>
+        <v>event_id</v>
+      </c>
+      <c r="B13" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C13" t="str">
+        <v>UUID of an event OR the word 'general' for homepage reviews.</v>
+      </c>
+      <c r="D13" t="str">
+        <v>3f2a1b4c-… OR general</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>── SHEET: Mapping (optional) ──────────────────────────────────────────</v>
+        <v>review_text</v>
+      </c>
+      <c r="B14" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C14" t="str">
+        <v>The full review text.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Amazing experience…</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Column</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Required?</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Description</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Example</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>review_id</v>
-      </c>
-      <c r="B16" t="str">
-        <v>YES</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Must exactly match a local_id from the Reviews sheet.</v>
-      </c>
-      <c r="D16" t="str">
-        <v>R1</v>
+        <v>── SHEET: Mapping (optional) ──────────────────────────────────────────</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>image_1</v>
+        <v>Column</v>
       </c>
       <c r="B17" t="str">
-        <v>NO</v>
+        <v>Required?</v>
       </c>
       <c r="C17" t="str">
-        <v>UUID of an image already uploaded via Admin → Images. Copy UUIDs from the 'Show uploaded image IDs' panel on the Imports page.</v>
+        <v>Description</v>
       </c>
       <c r="D17" t="str">
-        <v>a1b2c3d4-…</v>
+        <v>Example</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>image_2</v>
+        <v>review_id</v>
       </c>
       <c r="B18" t="str">
-        <v>NO</v>
+        <v>YES</v>
       </c>
       <c r="C18" t="str">
-        <v>Second image UUID (optional).</v>
+        <v>Must exactly match a local_id from the Reviews sheet.</v>
       </c>
       <c r="D18" t="str">
-        <v/>
+        <v>R1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>image_3</v>
+        <v>image_1</v>
       </c>
       <c r="B19" t="str">
         <v>NO</v>
       </c>
       <c r="C19" t="str">
-        <v>Third image UUID (optional, max 3 per review).</v>
+        <v>The TITLE of an image uploaded in Admin → Images. Case-insensitive.</v>
       </c>
       <c r="D19" t="str">
-        <v/>
+        <v>Beach Shot 1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v/>
+        <v>image_2</v>
+      </c>
+      <c r="B20" t="str">
+        <v>NO</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Second image title (optional).</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Group Photo</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>── REVIEW TYPE (auto-detected) ─────────────────────────────────────────</v>
+        <v>image_3</v>
+      </c>
+      <c r="B21" t="str">
+        <v>NO</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Third image title (optional, max 3 per review).</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v># images in Mapping</v>
-      </c>
-      <c r="B22" t="str">
-        <v>review_type that gets saved</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>0 — review has no row in Mapping, or all image columns blank</v>
-      </c>
-      <c r="B23" t="str">
-        <v>TEXT_ONLY</v>
+        <v>── REVIEW TYPE (auto-detected) ─────────────────────────────────────────</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>1</v>
+        <v># images in Mapping</v>
       </c>
       <c r="B24" t="str">
-        <v>SINGLE_IMAGE</v>
+        <v>review_type assigned</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2 or 3</v>
+        <v>0 (no row, or all image columns blank)</v>
       </c>
       <c r="B25" t="str">
-        <v>MULTI_IMAGE</v>
+        <v>TEXT_ONLY</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="B26" t="str">
+        <v>SINGLE_IMAGE</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>── RULES ───────────────────────────────────────────────────────────────</v>
+        <v>2 or 3</v>
+      </c>
+      <c r="B27" t="str">
+        <v>MULTI_IMAGE</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>✅ Each image UUID can only be assigned to ONE review. Duplicates are rejected.</v>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>✅ Images must be uploaded via Admin → Images before running the import.</v>
+        <v>── RULES ───────────────────────────────────────────────────────────────</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>✅ Copy image UUIDs from the Admin → Imports page — 'Show uploaded image IDs' panel.</v>
+        <v>✅ Upload images in Admin → Images BEFORE running the import.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>✅ Rows with errors are skipped; other rows still import successfully.</v>
+        <v>✅ Titles are matched case-insensitively: 'beach shot 1' = 'Beach Shot 1'.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>✅ The import is safe to re-run — failed rows can be fixed and retried.</v>
+        <v>✅ Each image can only be assigned to ONE review — duplicates are rejected.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>✅ event_id must be an exact UUID match or the literal word 'general'.</v>
+        <v>✅ Rows with errors are skipped; all other rows import successfully.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v/>
+        <v>✅ The import is safe to re-run after fixing errors.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>── USER EXPERIENCE ─────────────────────────────────────────────────────</v>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>When a review with photos is shown to a user, the photos appear below the review text.</v>
+        <v>── USER EXPERIENCE ─────────────────────────────────────────────────────</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>The user downloads the photos first, then clicks 'Post Review on Google'.</v>
+        <v>Photos linked to a review are shown below the review text when a user sees it.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Once they confirm the review was posted, the review AND all its linked photos are permanently retired (never shown again).</v>
+        <v>The user downloads the photos first, then posts the review on Google.</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Once posted, the review AND all its photos are permanently retired.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D39"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>